<commit_message>
docs: reconcile Epic 9 xlsx with Master/ledger (recover lost S9/S10 rows)
The Epic 9 Admin-Console source xlsx was stuck at 62 rows in git: the 12
S9/S10 rows (U10-09.1..6 + U10-10.1..6, all Done) were regenerated into
the Master Tracker + program ledger in 89dd758, but that commit captured a
stale copy of the epic's own xlsx — the staged change was lost when the
working tree was stashed/popped during the S9/S10 test-failure triage.

Working copy (74 rows, S9+S10 = 6/6 COMPLETE) already matches the committed
Master (Epic 9 = 74/74) and ledger; this just makes the epic's source file
consistent with them. No count change.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic9_Admin_Console.xlsx
+++ b/docs/DecisionOS_Epic9_Admin_Console.xlsx
@@ -498,7 +498,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -535,7 +534,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
@@ -548,7 +546,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -561,7 +558,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
@@ -574,7 +570,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
@@ -582,7 +577,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -614,7 +608,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -646,7 +639,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -678,7 +670,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
@@ -710,7 +701,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
@@ -742,7 +732,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
@@ -774,7 +763,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
@@ -806,7 +794,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
@@ -838,7 +825,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
@@ -870,7 +856,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
@@ -902,7 +887,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
@@ -974,7 +958,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Epic 9 IN PROGRESS. S0 shipped + S1-S8 COMPLETE (Tenant 360, impersonation, support desk, billing, observability, feature-flags/config, admin RBAC+2FA, announcements). 8 new admin tabs + a tenant announcement banner; 60+ new routes; route fingerprint tracked via the committed API-parity baseline. Browser preview QA: full 16-tab walk-through green after a motor aggregate() coroutine fix in admin_usage (see backlog U10-QA.1). Remaining: S9 (compliance/DPDP data ops) + S10 (admin polish, tests &amp; QA).</t>
+          <t>Epic 9 -- Admin / Platform Console COMPLETE. S0 shipped + S1-S10 done: Tenant 360, impersonation, support desk, billing, observability, feature-flags/config, admin RBAC+2FA, announcements, compliance &amp; data ops (DPDP export/retention/DSAR/erasure-receipt), and admin polish + a test &amp; parity gate. 10 admin tabs + a tenant announcement banner; ~68 admin routes, all behind the platform-admin gate.</t>
         </is>
       </c>
     </row>
@@ -1325,19 +1309,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
         <v>6</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1358,19 +1342,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D16" t="n">
         <v>6</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1390,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5099,6 +5083,666 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>U10-09.1</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>routers/admin_compliance.py</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>9</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Per-tenant data export API</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>GET /admin/tenants/{id}/export -- one JSON bundle of every tenant-scoped collection, built off the same TENANT_COLLECTIONS single-source-of-truth the deleter uses, so an export is a faithful pre-image of an erasure. Row-capped, audited.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>routers/admin_compliance.py :: admin_export_tenant</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>U10-09.2</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>services/retention.py + admin_compliance</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>9</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Retention policy + daily purge</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Per-tenant retention {enabled, ttl_days, collections} on transient/log collections only (activity, notifications, usage_events, wa_events, voice_notes, brain_audit, ingestions). MIN_TTL 30d guard. GET/PUT /admin/tenants/{id}/retention with dry-run candidate counts.</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>services/retention.py + admin_get/set_retention</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>U10-09.3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>routers/admin_compliance.py</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>9</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Consent + audit export</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>GET /admin/tenants/{id}/consent-export -- AI-processing consent state + consent-tagged activity + every platform-admin action targeting the tenant. The DPDP 'who agreed to what' trail.</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>admin_consent_export</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>U10-09.4</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>routers/admin_compliance.py</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>9</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Structured export-before-delete (erasure receipt)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>POST /admin/tenants/{id}/delete-with-export (super_admin) -- builds a full export bundle, THEN hard-deletes via admin_delete_tenant, returning the export as an erasure receipt + the deletion summary. DPDP 'documented deletion path', not just a delete button.</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>admin_delete_with_export</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>U10-09.5</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>routers/admin_compliance.py</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>9</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Per-user DSAR export</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>GET /admin/users/{id}/dsar -- data-subject-access-request: everything the platform holds about one person across the collections carrying a person-field (assignee_id/created_by/user_id/...).</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>admin_user_dsar</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>U10-09.6</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>workers/schedulers.py + admin_compliance</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>9</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Retention sweep: scheduler hook + manual trigger + status</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>run_retention_sweep wired into the leader-locked scheduler tick, throttled to once/~24h via a db.platform_ops marker. GET /admin/retention/status (all policies + candidates + last sweep) and POST /admin/retention/run (super_admin, dry-run default) for a manual purge.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>workers/schedulers._maybe_run_retention_sweep + admin_retention_status/run</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>U10-10.1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/admin/*</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>10</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Responsive admin + Compliance tab</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>New Compliance tab (Scales icon) with a responsive lg:grid-cols-2 layout: workspace search + data-subject actions on the left, platform retention sweep on the right. Tab nav already overflow-x scrolls; section grids collapse to one column on narrow viewports.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>frontend ComplianceSection.js + AdminPortal tab</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>U10-10.2</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>tests/test_admin_compliance.py</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>10</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>pytest for compliance endpoints</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Unit tests over a fake Mongo: retention policy resolution + defaults + MIN_TTL clamp, dry-run vs live purge and the &lt;cutoff window, disabled-policy no-op, cross-tenant isolation, sweep touches only policy tenants, and export covers TENANT_COLLECTIONS. 11 tests.</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>tests/test_admin_compliance.py</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>U10-10.3</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>tests/test_admin_rbac_matrix.py</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>10</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Admin RBAC matrix tests</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Exhaustive require_admin_role(*roles) matrix: super_admin passes every gate; a matching role passes; every other role is 403; read_only never reaches a mutating gate. Plus a check that the two destructive compliance routes are super_admin-only. 6 tests.</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>tests/test_admin_rbac_matrix.py</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>U10-10.4</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>tests/test_admin_parity.py</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>10</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Admin API-parity gate</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Focused /api/admin contract: every admin route resolves through get_platform_admin (allow-listing the open login + the tenant-owner audit-log path), all Sprint 9 compliance routes present, and the admin route count matches a committed number so an added/dropped admin route is an explicit diff.</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>tests/test_admin_parity.py</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>U10-10.5</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>cross-cutting (admin)</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>10</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Copy + UX consistency pass</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Compliance section reuses the shared admin dark-theme style consts (CARD/H2/H3/BTN/INP), mono uppercase labels, and semantic action colours (green export, red erasure, blue search) matching every other admin tab. Confirm dialogs name the blast radius on both irreversible actions.</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ComplianceSection styling + confirm copy</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>U10-10.6</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>cross-cutting (admin)</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>10</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Admin exit gate: whole-surface gate + parity</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>The admin-parity gate asserts NO /api/admin route is reachable without the platform-admin dependency (the security exit gate for a business-critical console) and the whole-app route baseline + fingerprint sha is regenerated to include the 8 new compliance routes. Full suite green.</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>test_admin_parity::test_every_admin_route_is_gated + regen'd api_route_baseline.json</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Epic 9 S9/S10 build 2026-08-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>